<commit_message>
New improvements related to the selectors
</commit_message>
<xml_diff>
--- a/Data/Temp/InvoicesReport UI Extraction.xlsx
+++ b/Data/Temp/InvoicesReport UI Extraction.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29930"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30002"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanielRicardoRochaQu\Downloads\Invoicing Bot\Recon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1220" documentId="13_ncr:1_{B5D6CEAF-E681-4588-8E6E-EF4492DB7BA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AA67935-33BF-47B8-AAB6-FA2AAFFD4CAE}"/>
+  <xr:revisionPtr revIDLastSave="1221" documentId="13_ncr:1_{B5D6CEAF-E681-4588-8E6E-EF4492DB7BA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1E9BAF7-DFE4-4C3B-83CC-F19F6A125004}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="6" activeTab="6" xr2:uid="{70E8A791-13CE-4BD4-B2C5-703777F4F9B6}"/>
   </bookViews>
@@ -1407,13 +1407,7 @@
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{665A5D82-60EC-45BF-9AFF-3D1DD22F2701}" name="Xero_Tax_Acc" displayName="Xero_Tax_Acc" ref="A1:F185" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="A1:F185" xr:uid="{665A5D82-60EC-45BF-9AFF-3D1DD22F2701}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Monthly Support Fee"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:F185" xr:uid="{665A5D82-60EC-45BF-9AFF-3D1DD22F2701}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{ADF06759-72AB-4C84-B20B-0E8D66CF7A70}" name="Line Item"/>
     <tableColumn id="4" xr3:uid="{136FB1F1-5689-4097-ACD2-3191F8E3FAEA}" name="Currency"/>
@@ -3451,7 +3445,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:6" hidden="1">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>72</v>
       </c>
@@ -3472,7 +3466,7 @@
         <v>FT Accountant - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="3" spans="1:6" hidden="1">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>74</v>
       </c>
@@ -3493,7 +3487,7 @@
         <v>FT Zoho Developer - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="4" spans="1:6" hidden="1">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>75</v>
       </c>
@@ -3514,7 +3508,7 @@
         <v>PT Wealth Management Paraplanner - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="5" spans="1:6" hidden="1">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>76</v>
       </c>
@@ -3535,7 +3529,7 @@
         <v>FT Salesforce Developer - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="6" spans="1:6" hidden="1">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>77</v>
       </c>
@@ -3556,7 +3550,7 @@
         <v>FT Wealth Management Paraplanner - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="7" spans="1:6" hidden="1">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>78</v>
       </c>
@@ -3577,7 +3571,7 @@
         <v>Full Stack Developer - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="8" spans="1:6" hidden="1">
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>79</v>
       </c>
@@ -3598,7 +3592,7 @@
         <v>Custom Service - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="9" spans="1:6" hidden="1">
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>80</v>
       </c>
@@ -3619,7 +3613,7 @@
         <v>PT Wealth Management Virtual Assistant - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="10" spans="1:6" hidden="1">
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>81</v>
       </c>
@@ -3640,7 +3634,7 @@
         <v>FT Bookkeeping - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="11" spans="1:6" hidden="1">
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>82</v>
       </c>
@@ -3661,7 +3655,7 @@
         <v>Oracle HCM Cloud Developer - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="12" spans="1:6" hidden="1">
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
         <v>83</v>
       </c>
@@ -3682,7 +3676,7 @@
         <v>PT Zoho Developer - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="13" spans="1:6" hidden="1">
+    <row r="13" spans="1:6">
       <c r="A13" t="s">
         <v>84</v>
       </c>
@@ -3703,7 +3697,7 @@
         <v>Full Time Custom Staff Aug - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="14" spans="1:6" hidden="1">
+    <row r="14" spans="1:6">
       <c r="A14" t="s">
         <v>85</v>
       </c>
@@ -3724,7 +3718,7 @@
         <v>Full Time Medical Staff - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="15" spans="1:6" hidden="1">
+    <row r="15" spans="1:6">
       <c r="A15" t="s">
         <v>86</v>
       </c>
@@ -3745,7 +3739,7 @@
         <v>Part Time Custom Staff Aug - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="16" spans="1:6" hidden="1">
+    <row r="16" spans="1:6">
       <c r="A16" t="s">
         <v>87</v>
       </c>
@@ -3766,7 +3760,7 @@
         <v>PT Accountant - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="17" spans="1:6" hidden="1">
+    <row r="17" spans="1:6">
       <c r="A17" t="s">
         <v>88</v>
       </c>
@@ -3787,7 +3781,7 @@
         <v>FT Wealth Management Virtual Assistant - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="18" spans="1:6" hidden="1">
+    <row r="18" spans="1:6">
       <c r="A18" t="s">
         <v>89</v>
       </c>
@@ -3808,7 +3802,7 @@
         <v>PT Bookkeeping - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="19" spans="1:6" hidden="1">
+    <row r="19" spans="1:6">
       <c r="A19" t="s">
         <v>90</v>
       </c>
@@ -3829,7 +3823,7 @@
         <v>Dedicated 24x7x365 Digital Assistant - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="20" spans="1:6" hidden="1">
+    <row r="20" spans="1:6">
       <c r="A20" t="s">
         <v>91</v>
       </c>
@@ -3850,7 +3844,7 @@
         <v>Data Analytics Managed Service - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="21" spans="1:6" hidden="1">
+    <row r="21" spans="1:6">
       <c r="A21" t="s">
         <v>92</v>
       </c>
@@ -3871,7 +3865,7 @@
         <v>Data Analytics Implementation - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="22" spans="1:6" hidden="1">
+    <row r="22" spans="1:6">
       <c r="A22" t="s">
         <v>93</v>
       </c>
@@ -3892,7 +3886,7 @@
         <v>FT RPA Developer - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="23" spans="1:6" hidden="1">
+    <row r="23" spans="1:6">
       <c r="A23" t="s">
         <v>94</v>
       </c>
@@ -3913,7 +3907,7 @@
         <v>DA Implementation Team - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="24" spans="1:6" hidden="1">
+    <row r="24" spans="1:6">
       <c r="A24" t="s">
         <v>95</v>
       </c>
@@ -3934,7 +3928,7 @@
         <v>AI Data Extraction per page - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="25" spans="1:6" hidden="1">
+    <row r="25" spans="1:6">
       <c r="A25" t="s">
         <v>96</v>
       </c>
@@ -3955,7 +3949,7 @@
         <v>Fractional Digital Assistant - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="26" spans="1:6" hidden="1">
+    <row r="26" spans="1:6">
       <c r="A26" t="s">
         <v>97</v>
       </c>
@@ -3976,7 +3970,7 @@
         <v>AI Workshop - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="27" spans="1:6" hidden="1">
+    <row r="27" spans="1:6">
       <c r="A27" t="s">
         <v>98</v>
       </c>
@@ -3997,7 +3991,7 @@
         <v>Background Verification Check Fee - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="28" spans="1:6" hidden="1">
+    <row r="28" spans="1:6">
       <c r="A28" t="s">
         <v>99</v>
       </c>
@@ -4018,7 +4012,7 @@
         <v>Onboarding Setup - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="29" spans="1:6" hidden="1">
+    <row r="29" spans="1:6">
       <c r="A29" t="s">
         <v>100</v>
       </c>
@@ -4039,7 +4033,7 @@
         <v>T&amp;M Staff Augmentation - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="30" spans="1:6" hidden="1">
+    <row r="30" spans="1:6">
       <c r="A30" t="s">
         <v>101</v>
       </c>
@@ -4060,7 +4054,7 @@
         <v>Custom Data Analytics Consulting - T&amp;M - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="31" spans="1:6" hidden="1">
+    <row r="31" spans="1:6">
       <c r="A31" t="s">
         <v>102</v>
       </c>
@@ -4081,7 +4075,7 @@
         <v>Data Analytics - Basic Maintenance - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="32" spans="1:6" hidden="1">
+    <row r="32" spans="1:6">
       <c r="A32" t="s">
         <v>103</v>
       </c>
@@ -4102,7 +4096,7 @@
         <v>Data Analytics - Light Managed Service - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="33" spans="1:6" hidden="1">
+    <row r="33" spans="1:6">
       <c r="A33" t="s">
         <v>104</v>
       </c>
@@ -4123,7 +4117,7 @@
         <v>Data Analytics - Managed Service - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="34" spans="1:6" hidden="1">
+    <row r="34" spans="1:6">
       <c r="A34" t="s">
         <v>105</v>
       </c>
@@ -4144,7 +4138,7 @@
         <v>Data Analytics - Prototype Model - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="35" spans="1:6" hidden="1">
+    <row r="35" spans="1:6">
       <c r="A35" t="s">
         <v>106</v>
       </c>
@@ -4165,7 +4159,7 @@
         <v>Reseller Monthly Fee - AUD - Reseller Pipeline</v>
       </c>
     </row>
-    <row r="36" spans="1:6" hidden="1">
+    <row r="36" spans="1:6">
       <c r="A36" t="s">
         <v>107</v>
       </c>
@@ -4186,7 +4180,7 @@
         <v>Franchise Setup Fee  - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="37" spans="1:6" hidden="1">
+    <row r="37" spans="1:6">
       <c r="A37" t="s">
         <v>108</v>
       </c>
@@ -4207,7 +4201,7 @@
         <v>Monthly Lead Gen Tech Stack Fee - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="38" spans="1:6" hidden="1">
+    <row r="38" spans="1:6">
       <c r="A38" t="s">
         <v>109</v>
       </c>
@@ -4249,7 +4243,7 @@
         <v>Monthly Support Fee - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="40" spans="1:6" hidden="1">
+    <row r="40" spans="1:6">
       <c r="A40" t="s">
         <v>111</v>
       </c>
@@ -4270,7 +4264,7 @@
         <v>Annual Conference Fee - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="41" spans="1:6" hidden="1">
+    <row r="41" spans="1:6">
       <c r="A41" t="s">
         <v>112</v>
       </c>
@@ -4291,7 +4285,7 @@
         <v>Monthly Consultant Access Fee - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="42" spans="1:6" hidden="1">
+    <row r="42" spans="1:6">
       <c r="A42" t="s">
         <v>113</v>
       </c>
@@ -4312,7 +4306,7 @@
         <v>COMPLEX - Ai Powered Data Extraction - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="43" spans="1:6" hidden="1">
+    <row r="43" spans="1:6">
       <c r="A43" t="s">
         <v>114</v>
       </c>
@@ -4333,7 +4327,7 @@
         <v>Ai Powered Data Extraction - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="44" spans="1:6" hidden="1">
+    <row r="44" spans="1:6">
       <c r="A44" t="s">
         <v>115</v>
       </c>
@@ -4354,7 +4348,7 @@
         <v>Digital Assistant - upto 250k Executions - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="45" spans="1:6" hidden="1">
+    <row r="45" spans="1:6">
       <c r="A45" t="s">
         <v>116</v>
       </c>
@@ -4375,7 +4369,7 @@
         <v>Digital Assistant - upto 100k Executions - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="46" spans="1:6" hidden="1">
+    <row r="46" spans="1:6">
       <c r="A46" t="s">
         <v>117</v>
       </c>
@@ -4396,7 +4390,7 @@
         <v>Digital Assistant - upto 50k Executions - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="47" spans="1:6" hidden="1">
+    <row r="47" spans="1:6">
       <c r="A47" t="s">
         <v>118</v>
       </c>
@@ -4417,7 +4411,7 @@
         <v>Digital Assistant - upto 10k Executions - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="48" spans="1:6" hidden="1">
+    <row r="48" spans="1:6">
       <c r="A48" t="s">
         <v>119</v>
       </c>
@@ -4438,7 +4432,7 @@
         <v>MSP Reseller - AUD - MSP Pipeline</v>
       </c>
     </row>
-    <row r="49" spans="1:6" hidden="1">
+    <row r="49" spans="1:6">
       <c r="A49" t="s">
         <v>121</v>
       </c>
@@ -4459,7 +4453,7 @@
         <v>MSP Referral Partner - AUD - MSP Pipeline</v>
       </c>
     </row>
-    <row r="50" spans="1:6" hidden="1">
+    <row r="50" spans="1:6">
       <c r="A50" t="s">
         <v>122</v>
       </c>
@@ -4480,7 +4474,7 @@
         <v>MSP Service Delivery Partner - AUD - MSP Pipeline</v>
       </c>
     </row>
-    <row r="51" spans="1:6" hidden="1">
+    <row r="51" spans="1:6">
       <c r="A51" t="s">
         <v>72</v>
       </c>
@@ -4501,7 +4495,7 @@
         <v>FT Accountant - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="52" spans="1:6" hidden="1">
+    <row r="52" spans="1:6">
       <c r="A52" t="s">
         <v>74</v>
       </c>
@@ -4522,7 +4516,7 @@
         <v>FT Zoho Developer - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="53" spans="1:6" hidden="1">
+    <row r="53" spans="1:6">
       <c r="A53" t="s">
         <v>75</v>
       </c>
@@ -4543,7 +4537,7 @@
         <v>PT Wealth Management Paraplanner - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="54" spans="1:6" hidden="1">
+    <row r="54" spans="1:6">
       <c r="A54" t="s">
         <v>76</v>
       </c>
@@ -4564,7 +4558,7 @@
         <v>FT Salesforce Developer - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="55" spans="1:6" hidden="1">
+    <row r="55" spans="1:6">
       <c r="A55" t="s">
         <v>77</v>
       </c>
@@ -4585,7 +4579,7 @@
         <v>FT Wealth Management Paraplanner - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="56" spans="1:6" hidden="1">
+    <row r="56" spans="1:6">
       <c r="A56" t="s">
         <v>78</v>
       </c>
@@ -4606,7 +4600,7 @@
         <v>Full Stack Developer - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="57" spans="1:6" hidden="1">
+    <row r="57" spans="1:6">
       <c r="A57" t="s">
         <v>79</v>
       </c>
@@ -4627,7 +4621,7 @@
         <v>Custom Service - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="58" spans="1:6" hidden="1">
+    <row r="58" spans="1:6">
       <c r="A58" t="s">
         <v>80</v>
       </c>
@@ -4648,7 +4642,7 @@
         <v>PT Wealth Management Virtual Assistant - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="59" spans="1:6" hidden="1">
+    <row r="59" spans="1:6">
       <c r="A59" t="s">
         <v>81</v>
       </c>
@@ -4669,7 +4663,7 @@
         <v>FT Bookkeeping - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="60" spans="1:6" hidden="1">
+    <row r="60" spans="1:6">
       <c r="A60" t="s">
         <v>82</v>
       </c>
@@ -4690,7 +4684,7 @@
         <v>Oracle HCM Cloud Developer - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="61" spans="1:6" hidden="1">
+    <row r="61" spans="1:6">
       <c r="A61" t="s">
         <v>83</v>
       </c>
@@ -4711,7 +4705,7 @@
         <v>PT Zoho Developer - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="62" spans="1:6" hidden="1">
+    <row r="62" spans="1:6">
       <c r="A62" t="s">
         <v>84</v>
       </c>
@@ -4732,7 +4726,7 @@
         <v>Full Time Custom Staff Aug - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="63" spans="1:6" hidden="1">
+    <row r="63" spans="1:6">
       <c r="A63" t="s">
         <v>85</v>
       </c>
@@ -4753,7 +4747,7 @@
         <v>Full Time Medical Staff - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="64" spans="1:6" hidden="1">
+    <row r="64" spans="1:6">
       <c r="A64" t="s">
         <v>86</v>
       </c>
@@ -4774,7 +4768,7 @@
         <v>Part Time Custom Staff Aug - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="65" spans="1:6" hidden="1">
+    <row r="65" spans="1:6">
       <c r="A65" t="s">
         <v>87</v>
       </c>
@@ -4795,7 +4789,7 @@
         <v>PT Accountant - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="66" spans="1:6" hidden="1">
+    <row r="66" spans="1:6">
       <c r="A66" t="s">
         <v>88</v>
       </c>
@@ -4816,7 +4810,7 @@
         <v>FT Wealth Management Virtual Assistant - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="67" spans="1:6" hidden="1">
+    <row r="67" spans="1:6">
       <c r="A67" t="s">
         <v>89</v>
       </c>
@@ -4837,7 +4831,7 @@
         <v>PT Bookkeeping - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="68" spans="1:6" hidden="1">
+    <row r="68" spans="1:6">
       <c r="A68" t="s">
         <v>90</v>
       </c>
@@ -4858,7 +4852,7 @@
         <v>Dedicated 24x7x365 Digital Assistant - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="69" spans="1:6" hidden="1">
+    <row r="69" spans="1:6">
       <c r="A69" t="s">
         <v>91</v>
       </c>
@@ -4879,7 +4873,7 @@
         <v>Data Analytics Managed Service - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="70" spans="1:6" hidden="1">
+    <row r="70" spans="1:6">
       <c r="A70" t="s">
         <v>92</v>
       </c>
@@ -4900,7 +4894,7 @@
         <v>Data Analytics Implementation - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="71" spans="1:6" hidden="1">
+    <row r="71" spans="1:6">
       <c r="A71" t="s">
         <v>93</v>
       </c>
@@ -4921,7 +4915,7 @@
         <v>FT RPA Developer - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="72" spans="1:6" hidden="1">
+    <row r="72" spans="1:6">
       <c r="A72" t="s">
         <v>94</v>
       </c>
@@ -4942,7 +4936,7 @@
         <v>DA Implementation Team - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="73" spans="1:6" hidden="1">
+    <row r="73" spans="1:6">
       <c r="A73" t="s">
         <v>95</v>
       </c>
@@ -4963,7 +4957,7 @@
         <v>AI Data Extraction per page - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="74" spans="1:6" hidden="1">
+    <row r="74" spans="1:6">
       <c r="A74" t="s">
         <v>96</v>
       </c>
@@ -4984,7 +4978,7 @@
         <v>Fractional Digital Assistant - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="75" spans="1:6" hidden="1">
+    <row r="75" spans="1:6">
       <c r="A75" t="s">
         <v>97</v>
       </c>
@@ -5005,7 +4999,7 @@
         <v>AI Workshop - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="76" spans="1:6" hidden="1">
+    <row r="76" spans="1:6">
       <c r="A76" t="s">
         <v>98</v>
       </c>
@@ -5026,7 +5020,7 @@
         <v>Background Verification Check Fee - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="77" spans="1:6" hidden="1">
+    <row r="77" spans="1:6">
       <c r="A77" t="s">
         <v>99</v>
       </c>
@@ -5047,7 +5041,7 @@
         <v>Onboarding Setup - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="78" spans="1:6" hidden="1">
+    <row r="78" spans="1:6">
       <c r="A78" t="s">
         <v>100</v>
       </c>
@@ -5068,7 +5062,7 @@
         <v>T&amp;M Staff Augmentation - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="79" spans="1:6" hidden="1">
+    <row r="79" spans="1:6">
       <c r="A79" t="s">
         <v>101</v>
       </c>
@@ -5089,7 +5083,7 @@
         <v>Custom Data Analytics Consulting - T&amp;M - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="80" spans="1:6" hidden="1">
+    <row r="80" spans="1:6">
       <c r="A80" t="s">
         <v>102</v>
       </c>
@@ -5110,7 +5104,7 @@
         <v>Data Analytics - Basic Maintenance - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="81" spans="1:6" hidden="1">
+    <row r="81" spans="1:6">
       <c r="A81" t="s">
         <v>103</v>
       </c>
@@ -5131,7 +5125,7 @@
         <v>Data Analytics - Light Managed Service - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="82" spans="1:6" hidden="1">
+    <row r="82" spans="1:6">
       <c r="A82" t="s">
         <v>104</v>
       </c>
@@ -5152,7 +5146,7 @@
         <v>Data Analytics - Managed Service - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="83" spans="1:6" hidden="1">
+    <row r="83" spans="1:6">
       <c r="A83" t="s">
         <v>105</v>
       </c>
@@ -5173,7 +5167,7 @@
         <v>Data Analytics - Prototype Model - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="84" spans="1:6" hidden="1">
+    <row r="84" spans="1:6">
       <c r="A84" t="s">
         <v>106</v>
       </c>
@@ -5194,7 +5188,7 @@
         <v>Reseller Monthly Fee - NZD - Reseller Pipeline</v>
       </c>
     </row>
-    <row r="85" spans="1:6" hidden="1">
+    <row r="85" spans="1:6">
       <c r="A85" t="s">
         <v>107</v>
       </c>
@@ -5215,7 +5209,7 @@
         <v>Franchise Setup Fee  - NZD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="86" spans="1:6" hidden="1">
+    <row r="86" spans="1:6">
       <c r="A86" t="s">
         <v>108</v>
       </c>
@@ -5236,7 +5230,7 @@
         <v>Monthly Lead Gen Tech Stack Fee - NZD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="87" spans="1:6" hidden="1">
+    <row r="87" spans="1:6">
       <c r="A87" t="s">
         <v>109</v>
       </c>
@@ -5278,7 +5272,7 @@
         <v>Monthly Support Fee - NZD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="89" spans="1:6" hidden="1">
+    <row r="89" spans="1:6">
       <c r="A89" t="s">
         <v>111</v>
       </c>
@@ -5299,7 +5293,7 @@
         <v>Annual Conference Fee - NZD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="90" spans="1:6" hidden="1">
+    <row r="90" spans="1:6">
       <c r="A90" t="s">
         <v>112</v>
       </c>
@@ -5320,7 +5314,7 @@
         <v>Monthly Consultant Access Fee - NZD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="91" spans="1:6" hidden="1">
+    <row r="91" spans="1:6">
       <c r="A91" t="s">
         <v>113</v>
       </c>
@@ -5341,7 +5335,7 @@
         <v>COMPLEX - Ai Powered Data Extraction - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="92" spans="1:6" hidden="1">
+    <row r="92" spans="1:6">
       <c r="A92" t="s">
         <v>114</v>
       </c>
@@ -5362,7 +5356,7 @@
         <v>Ai Powered Data Extraction - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="93" spans="1:6" hidden="1">
+    <row r="93" spans="1:6">
       <c r="A93" t="s">
         <v>115</v>
       </c>
@@ -5383,7 +5377,7 @@
         <v>Digital Assistant - upto 250k Executions - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="94" spans="1:6" hidden="1">
+    <row r="94" spans="1:6">
       <c r="A94" t="s">
         <v>116</v>
       </c>
@@ -5404,7 +5398,7 @@
         <v>Digital Assistant - upto 100k Executions - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="95" spans="1:6" hidden="1">
+    <row r="95" spans="1:6">
       <c r="A95" t="s">
         <v>117</v>
       </c>
@@ -5425,7 +5419,7 @@
         <v>Digital Assistant - upto 50k Executions - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="96" spans="1:6" hidden="1">
+    <row r="96" spans="1:6">
       <c r="A96" t="s">
         <v>118</v>
       </c>
@@ -5446,7 +5440,7 @@
         <v>Digital Assistant - upto 10k Executions - NZD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="97" spans="1:6" hidden="1">
+    <row r="97" spans="1:6">
       <c r="A97" t="s">
         <v>119</v>
       </c>
@@ -5467,7 +5461,7 @@
         <v>MSP Reseller - NZD - MSP Pipeline</v>
       </c>
     </row>
-    <row r="98" spans="1:6" hidden="1">
+    <row r="98" spans="1:6">
       <c r="A98" t="s">
         <v>121</v>
       </c>
@@ -5488,7 +5482,7 @@
         <v>MSP Referral Partner - NZD - MSP Pipeline</v>
       </c>
     </row>
-    <row r="99" spans="1:6" hidden="1">
+    <row r="99" spans="1:6">
       <c r="A99" t="s">
         <v>122</v>
       </c>
@@ -5509,7 +5503,7 @@
         <v>MSP Service Delivery Partner - NZD - MSP Pipeline</v>
       </c>
     </row>
-    <row r="100" spans="1:6" hidden="1">
+    <row r="100" spans="1:6">
       <c r="A100" t="s">
         <v>72</v>
       </c>
@@ -5530,7 +5524,7 @@
         <v>FT Accountant - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="101" spans="1:6" hidden="1">
+    <row r="101" spans="1:6">
       <c r="A101" t="s">
         <v>74</v>
       </c>
@@ -5551,7 +5545,7 @@
         <v>FT Zoho Developer - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="102" spans="1:6" hidden="1">
+    <row r="102" spans="1:6">
       <c r="A102" t="s">
         <v>75</v>
       </c>
@@ -5572,7 +5566,7 @@
         <v>PT Wealth Management Paraplanner - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="103" spans="1:6" hidden="1">
+    <row r="103" spans="1:6">
       <c r="A103" t="s">
         <v>76</v>
       </c>
@@ -5593,7 +5587,7 @@
         <v>FT Salesforce Developer - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="104" spans="1:6" hidden="1">
+    <row r="104" spans="1:6">
       <c r="A104" t="s">
         <v>77</v>
       </c>
@@ -5614,7 +5608,7 @@
         <v>FT Wealth Management Paraplanner - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="105" spans="1:6" hidden="1">
+    <row r="105" spans="1:6">
       <c r="A105" t="s">
         <v>78</v>
       </c>
@@ -5635,7 +5629,7 @@
         <v>Full Stack Developer - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="106" spans="1:6" hidden="1">
+    <row r="106" spans="1:6">
       <c r="A106" t="s">
         <v>79</v>
       </c>
@@ -5656,7 +5650,7 @@
         <v>Custom Service - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="107" spans="1:6" hidden="1">
+    <row r="107" spans="1:6">
       <c r="A107" t="s">
         <v>80</v>
       </c>
@@ -5677,7 +5671,7 @@
         <v>PT Wealth Management Virtual Assistant - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="108" spans="1:6" hidden="1">
+    <row r="108" spans="1:6">
       <c r="A108" t="s">
         <v>81</v>
       </c>
@@ -5698,7 +5692,7 @@
         <v>FT Bookkeeping - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="109" spans="1:6" hidden="1">
+    <row r="109" spans="1:6">
       <c r="A109" t="s">
         <v>82</v>
       </c>
@@ -5719,7 +5713,7 @@
         <v>Oracle HCM Cloud Developer - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="110" spans="1:6" hidden="1">
+    <row r="110" spans="1:6">
       <c r="A110" t="s">
         <v>83</v>
       </c>
@@ -5740,7 +5734,7 @@
         <v>PT Zoho Developer - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="111" spans="1:6" hidden="1">
+    <row r="111" spans="1:6">
       <c r="A111" t="s">
         <v>84</v>
       </c>
@@ -5761,7 +5755,7 @@
         <v>Full Time Custom Staff Aug - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="112" spans="1:6" hidden="1">
+    <row r="112" spans="1:6">
       <c r="A112" t="s">
         <v>85</v>
       </c>
@@ -5782,7 +5776,7 @@
         <v>Full Time Medical Staff - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="113" spans="1:6" hidden="1">
+    <row r="113" spans="1:6">
       <c r="A113" t="s">
         <v>86</v>
       </c>
@@ -5803,7 +5797,7 @@
         <v>Part Time Custom Staff Aug - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="114" spans="1:6" hidden="1">
+    <row r="114" spans="1:6">
       <c r="A114" t="s">
         <v>87</v>
       </c>
@@ -5824,7 +5818,7 @@
         <v>PT Accountant - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="115" spans="1:6" hidden="1">
+    <row r="115" spans="1:6">
       <c r="A115" t="s">
         <v>88</v>
       </c>
@@ -5845,7 +5839,7 @@
         <v>FT Wealth Management Virtual Assistant - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="116" spans="1:6" hidden="1">
+    <row r="116" spans="1:6">
       <c r="A116" t="s">
         <v>89</v>
       </c>
@@ -5866,7 +5860,7 @@
         <v>PT Bookkeeping - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="117" spans="1:6" hidden="1">
+    <row r="117" spans="1:6">
       <c r="A117" t="s">
         <v>90</v>
       </c>
@@ -5887,7 +5881,7 @@
         <v>Dedicated 24x7x365 Digital Assistant - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="118" spans="1:6" hidden="1">
+    <row r="118" spans="1:6">
       <c r="A118" t="s">
         <v>91</v>
       </c>
@@ -5908,7 +5902,7 @@
         <v>Data Analytics Managed Service - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="119" spans="1:6" hidden="1">
+    <row r="119" spans="1:6">
       <c r="A119" t="s">
         <v>92</v>
       </c>
@@ -5929,7 +5923,7 @@
         <v>Data Analytics Implementation - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="120" spans="1:6" hidden="1">
+    <row r="120" spans="1:6">
       <c r="A120" t="s">
         <v>93</v>
       </c>
@@ -5950,7 +5944,7 @@
         <v>FT RPA Developer - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="121" spans="1:6" hidden="1">
+    <row r="121" spans="1:6">
       <c r="A121" t="s">
         <v>94</v>
       </c>
@@ -5971,7 +5965,7 @@
         <v>DA Implementation Team - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="122" spans="1:6" hidden="1">
+    <row r="122" spans="1:6">
       <c r="A122" t="s">
         <v>95</v>
       </c>
@@ -5992,7 +5986,7 @@
         <v>AI Data Extraction per page - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="123" spans="1:6" hidden="1">
+    <row r="123" spans="1:6">
       <c r="A123" t="s">
         <v>96</v>
       </c>
@@ -6013,7 +6007,7 @@
         <v>Fractional Digital Assistant - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="124" spans="1:6" hidden="1">
+    <row r="124" spans="1:6">
       <c r="A124" t="s">
         <v>97</v>
       </c>
@@ -6034,7 +6028,7 @@
         <v>AI Workshop - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="125" spans="1:6" hidden="1">
+    <row r="125" spans="1:6">
       <c r="A125" t="s">
         <v>98</v>
       </c>
@@ -6055,7 +6049,7 @@
         <v>Background Verification Check Fee - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="126" spans="1:6" hidden="1">
+    <row r="126" spans="1:6">
       <c r="A126" t="s">
         <v>99</v>
       </c>
@@ -6076,7 +6070,7 @@
         <v>Onboarding Setup - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="127" spans="1:6" hidden="1">
+    <row r="127" spans="1:6">
       <c r="A127" t="s">
         <v>100</v>
       </c>
@@ -6097,7 +6091,7 @@
         <v>T&amp;M Staff Augmentation - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="128" spans="1:6" hidden="1">
+    <row r="128" spans="1:6">
       <c r="A128" t="s">
         <v>101</v>
       </c>
@@ -6118,7 +6112,7 @@
         <v>Custom Data Analytics Consulting - T&amp;M - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="129" spans="1:6" hidden="1">
+    <row r="129" spans="1:6">
       <c r="A129" t="s">
         <v>102</v>
       </c>
@@ -6139,7 +6133,7 @@
         <v>Data Analytics - Basic Maintenance - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="130" spans="1:6" hidden="1">
+    <row r="130" spans="1:6">
       <c r="A130" t="s">
         <v>103</v>
       </c>
@@ -6160,7 +6154,7 @@
         <v>Data Analytics - Light Managed Service - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="131" spans="1:6" hidden="1">
+    <row r="131" spans="1:6">
       <c r="A131" t="s">
         <v>104</v>
       </c>
@@ -6181,7 +6175,7 @@
         <v>Data Analytics - Managed Service - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="132" spans="1:6" hidden="1">
+    <row r="132" spans="1:6">
       <c r="A132" t="s">
         <v>105</v>
       </c>
@@ -6202,7 +6196,7 @@
         <v>Data Analytics - Prototype Model - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="133" spans="1:6" hidden="1">
+    <row r="133" spans="1:6">
       <c r="A133" t="s">
         <v>106</v>
       </c>
@@ -6223,7 +6217,7 @@
         <v>Reseller Monthly Fee - GBP - Reseller Pipeline</v>
       </c>
     </row>
-    <row r="134" spans="1:6" hidden="1">
+    <row r="134" spans="1:6">
       <c r="A134" t="s">
         <v>107</v>
       </c>
@@ -6244,7 +6238,7 @@
         <v>Franchise Setup Fee  - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="135" spans="1:6" hidden="1">
+    <row r="135" spans="1:6">
       <c r="A135" t="s">
         <v>108</v>
       </c>
@@ -6265,7 +6259,7 @@
         <v>Monthly Lead Gen Tech Stack Fee - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="136" spans="1:6" hidden="1">
+    <row r="136" spans="1:6">
       <c r="A136" t="s">
         <v>109</v>
       </c>
@@ -6307,7 +6301,7 @@
         <v>Monthly Support Fee - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="138" spans="1:6" hidden="1">
+    <row r="138" spans="1:6">
       <c r="A138" t="s">
         <v>111</v>
       </c>
@@ -6328,7 +6322,7 @@
         <v>Annual Conference Fee - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="139" spans="1:6" hidden="1">
+    <row r="139" spans="1:6">
       <c r="A139" t="s">
         <v>112</v>
       </c>
@@ -6349,7 +6343,7 @@
         <v>Monthly Consultant Access Fee - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="140" spans="1:6" hidden="1">
+    <row r="140" spans="1:6">
       <c r="A140" t="s">
         <v>113</v>
       </c>
@@ -6370,7 +6364,7 @@
         <v>COMPLEX - Ai Powered Data Extraction - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="141" spans="1:6" hidden="1">
+    <row r="141" spans="1:6">
       <c r="A141" t="s">
         <v>114</v>
       </c>
@@ -6391,7 +6385,7 @@
         <v>Ai Powered Data Extraction - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="142" spans="1:6" hidden="1">
+    <row r="142" spans="1:6">
       <c r="A142" t="s">
         <v>115</v>
       </c>
@@ -6412,7 +6406,7 @@
         <v>Digital Assistant - upto 250k Executions - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="143" spans="1:6" hidden="1">
+    <row r="143" spans="1:6">
       <c r="A143" t="s">
         <v>116</v>
       </c>
@@ -6433,7 +6427,7 @@
         <v>Digital Assistant - upto 100k Executions - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="144" spans="1:6" hidden="1">
+    <row r="144" spans="1:6">
       <c r="A144" t="s">
         <v>117</v>
       </c>
@@ -6454,7 +6448,7 @@
         <v>Digital Assistant - upto 50k Executions - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="145" spans="1:6" hidden="1">
+    <row r="145" spans="1:6">
       <c r="A145" t="s">
         <v>118</v>
       </c>
@@ -6475,7 +6469,7 @@
         <v>Digital Assistant - upto 10k Executions - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="146" spans="1:6" hidden="1">
+    <row r="146" spans="1:6">
       <c r="A146" t="s">
         <v>119</v>
       </c>
@@ -6496,7 +6490,7 @@
         <v>MSP Reseller - GBP - MSP Pipeline</v>
       </c>
     </row>
-    <row r="147" spans="1:6" hidden="1">
+    <row r="147" spans="1:6">
       <c r="A147" t="s">
         <v>121</v>
       </c>
@@ -6517,7 +6511,7 @@
         <v>MSP Referral Partner - GBP - MSP Pipeline</v>
       </c>
     </row>
-    <row r="148" spans="1:6" hidden="1">
+    <row r="148" spans="1:6">
       <c r="A148" t="s">
         <v>122</v>
       </c>
@@ -6538,7 +6532,7 @@
         <v>MSP Service Delivery Partner - GBP - MSP Pipeline</v>
       </c>
     </row>
-    <row r="149" spans="1:6" hidden="1">
+    <row r="149" spans="1:6">
       <c r="A149" t="s">
         <v>126</v>
       </c>
@@ -6559,7 +6553,7 @@
         <v>Consultant - Dripify License - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="150" spans="1:6" hidden="1">
+    <row r="150" spans="1:6">
       <c r="A150" t="s">
         <v>127</v>
       </c>
@@ -6580,7 +6574,7 @@
         <v>1Password License - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="151" spans="1:6" hidden="1">
+    <row r="151" spans="1:6">
       <c r="A151" t="s">
         <v>128</v>
       </c>
@@ -6601,7 +6595,7 @@
         <v>Consultant - MS Email Only + 1Password - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="152" spans="1:6" hidden="1">
+    <row r="152" spans="1:6">
       <c r="A152" t="s">
         <v>129</v>
       </c>
@@ -6622,7 +6616,7 @@
         <v>Consultant - HubSpot Sales License - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="153" spans="1:6" hidden="1">
+    <row r="153" spans="1:6">
       <c r="A153" t="s">
         <v>130</v>
       </c>
@@ -6643,7 +6637,7 @@
         <v>Consultant - MS CoPilot License - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="154" spans="1:6" hidden="1">
+    <row r="154" spans="1:6">
       <c r="A154" t="s">
         <v>131</v>
       </c>
@@ -6664,7 +6658,7 @@
         <v>HubSpot Sales License - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="155" spans="1:6" hidden="1">
+    <row r="155" spans="1:6">
       <c r="A155" t="s">
         <v>132</v>
       </c>
@@ -6685,7 +6679,7 @@
         <v>Consultant - Apollo License - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="156" spans="1:6" hidden="1">
+    <row r="156" spans="1:6">
       <c r="A156" t="s">
         <v>133</v>
       </c>
@@ -6706,7 +6700,7 @@
         <v>Consultant - MS Email Only - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="157" spans="1:6" hidden="1">
+    <row r="157" spans="1:6">
       <c r="A157" t="s">
         <v>134</v>
       </c>
@@ -6727,7 +6721,7 @@
         <v>Consultant - MS O365 License + 1Password - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="158" spans="1:6" hidden="1">
+    <row r="158" spans="1:6">
       <c r="A158" t="s">
         <v>135</v>
       </c>
@@ -6748,7 +6742,7 @@
         <v>Dripify License - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="159" spans="1:6" hidden="1">
+    <row r="159" spans="1:6">
       <c r="A159" t="s">
         <v>136</v>
       </c>
@@ -6769,7 +6763,7 @@
         <v>Monthly Annual Conference Fee - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="160" spans="1:6" hidden="1">
+    <row r="160" spans="1:6">
       <c r="A160" t="s">
         <v>137</v>
       </c>
@@ -6790,7 +6784,7 @@
         <v>MS CoPilot License - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="161" spans="1:6" hidden="1">
+    <row r="161" spans="1:6">
       <c r="A161" t="s">
         <v>138</v>
       </c>
@@ -6811,7 +6805,7 @@
         <v>MS O365 License + 1Password - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="162" spans="1:6" hidden="1">
+    <row r="162" spans="1:6">
       <c r="A162" t="s">
         <v>139</v>
       </c>
@@ -6832,7 +6826,7 @@
         <v>Apollo License - AUD - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="163" spans="1:6" hidden="1">
+    <row r="163" spans="1:6">
       <c r="A163" t="s">
         <v>140</v>
       </c>
@@ -6853,7 +6847,7 @@
         <v>Data Analyst - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="164" spans="1:6" hidden="1">
+    <row r="164" spans="1:6">
       <c r="A164" t="s">
         <v>141</v>
       </c>
@@ -6874,7 +6868,7 @@
         <v>Reseller International - AUD - Reseller Pipeline</v>
       </c>
     </row>
-    <row r="165" spans="1:6" hidden="1">
+    <row r="165" spans="1:6">
       <c r="A165" t="s">
         <v>106</v>
       </c>
@@ -6895,7 +6889,7 @@
         <v>Reseller Monthly Fee - AUD - Reseller Pipeline</v>
       </c>
     </row>
-    <row r="166" spans="1:6" hidden="1">
+    <row r="166" spans="1:6">
       <c r="A166" t="s">
         <v>126</v>
       </c>
@@ -6916,7 +6910,7 @@
         <v>Consultant - Dripify License - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="167" spans="1:6" hidden="1">
+    <row r="167" spans="1:6">
       <c r="A167" t="s">
         <v>127</v>
       </c>
@@ -6937,7 +6931,7 @@
         <v>1Password License - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="168" spans="1:6" hidden="1">
+    <row r="168" spans="1:6">
       <c r="A168" t="s">
         <v>128</v>
       </c>
@@ -6958,7 +6952,7 @@
         <v>Consultant - MS Email Only + 1Password - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="169" spans="1:6" hidden="1">
+    <row r="169" spans="1:6">
       <c r="A169" t="s">
         <v>129</v>
       </c>
@@ -6979,7 +6973,7 @@
         <v>Consultant - HubSpot Sales License - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="170" spans="1:6" hidden="1">
+    <row r="170" spans="1:6">
       <c r="A170" t="s">
         <v>130</v>
       </c>
@@ -7000,7 +6994,7 @@
         <v>Consultant - MS CoPilot License - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="171" spans="1:6" hidden="1">
+    <row r="171" spans="1:6">
       <c r="A171" t="s">
         <v>131</v>
       </c>
@@ -7021,7 +7015,7 @@
         <v>HubSpot Sales License - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="172" spans="1:6" hidden="1">
+    <row r="172" spans="1:6">
       <c r="A172" t="s">
         <v>132</v>
       </c>
@@ -7042,7 +7036,7 @@
         <v>Consultant - Apollo License - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="173" spans="1:6" hidden="1">
+    <row r="173" spans="1:6">
       <c r="A173" t="s">
         <v>133</v>
       </c>
@@ -7063,7 +7057,7 @@
         <v>Consultant - MS Email Only - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="174" spans="1:6" hidden="1">
+    <row r="174" spans="1:6">
       <c r="A174" t="s">
         <v>134</v>
       </c>
@@ -7084,7 +7078,7 @@
         <v>Consultant - MS O365 License + 1Password - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="175" spans="1:6" hidden="1">
+    <row r="175" spans="1:6">
       <c r="A175" t="s">
         <v>135</v>
       </c>
@@ -7105,7 +7099,7 @@
         <v>Dripify License - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="176" spans="1:6" hidden="1">
+    <row r="176" spans="1:6">
       <c r="A176" t="s">
         <v>136</v>
       </c>
@@ -7126,7 +7120,7 @@
         <v>Monthly Annual Conference Fee - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="177" spans="1:6" hidden="1">
+    <row r="177" spans="1:6">
       <c r="A177" t="s">
         <v>137</v>
       </c>
@@ -7147,7 +7141,7 @@
         <v>MS CoPilot License - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="178" spans="1:6" hidden="1">
+    <row r="178" spans="1:6">
       <c r="A178" t="s">
         <v>138</v>
       </c>
@@ -7168,7 +7162,7 @@
         <v>MS O365 License + 1Password - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="179" spans="1:6" hidden="1">
+    <row r="179" spans="1:6">
       <c r="A179" t="s">
         <v>139</v>
       </c>
@@ -7189,7 +7183,7 @@
         <v>Apollo License - GBP - Franchise Pipeline</v>
       </c>
     </row>
-    <row r="180" spans="1:6" hidden="1">
+    <row r="180" spans="1:6">
       <c r="A180" t="s">
         <v>140</v>
       </c>
@@ -7210,7 +7204,7 @@
         <v>Data Analyst - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="181" spans="1:6" hidden="1">
+    <row r="181" spans="1:6">
       <c r="A181" t="s">
         <v>141</v>
       </c>
@@ -7231,7 +7225,7 @@
         <v>Reseller International - GBP - Reseller Pipeline</v>
       </c>
     </row>
-    <row r="182" spans="1:6" hidden="1">
+    <row r="182" spans="1:6">
       <c r="A182" t="s">
         <v>142</v>
       </c>
@@ -7252,7 +7246,7 @@
         <v>Client Staff Bonus - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="183" spans="1:6" hidden="1">
+    <row r="183" spans="1:6">
       <c r="A183" t="s">
         <v>142</v>
       </c>
@@ -7273,7 +7267,7 @@
         <v>Client Staff Bonus - GBP - Sales Pipeline</v>
       </c>
     </row>
-    <row r="184" spans="1:6" hidden="1">
+    <row r="184" spans="1:6">
       <c r="A184" t="s">
         <v>145</v>
       </c>
@@ -7294,7 +7288,7 @@
         <v>Staff Aug 1.5x Project - AUD - Sales Pipeline</v>
       </c>
     </row>
-    <row r="185" spans="1:6" hidden="1">
+    <row r="185" spans="1:6">
       <c r="A185" t="s">
         <v>145</v>
       </c>
@@ -7324,6 +7318,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="2b4b3f37-1cd0-4b26-90f2-9948314503a5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca9c0abd-4151-432c-97d3-4a3f10bfee7f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005F54BCC7603DAA4FB57C31851CA92685" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b666b694d6e76699e884a198b0fcc20b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ca9c0abd-4151-432c-97d3-4a3f10bfee7f" xmlns:ns3="2b4b3f37-1cd0-4b26-90f2-9948314503a5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3e06c0a76cf39f93bdfa440a1b88f7bb" ns2:_="" ns3:_="">
     <xsd:import namespace="ca9c0abd-4151-432c-97d3-4a3f10bfee7f"/>
@@ -7564,28 +7578,8 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="2b4b3f37-1cd0-4b26-90f2-9948314503a5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ca9c0abd-4151-432c-97d3-4a3f10bfee7f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0554FEC5-F8C0-4A0B-9C72-9FC3334369E2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D60A3338-C622-4FF5-BFA9-54DFDA479994}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7593,5 +7587,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D60A3338-C622-4FF5-BFA9-54DFDA479994}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0554FEC5-F8C0-4A0B-9C72-9FC3334369E2}"/>
 </file>
</xml_diff>